<commit_message>
update, reportes y bugs de notificaciones
</commit_message>
<xml_diff>
--- a/R.Empresa.xlsx
+++ b/R.Empresa.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="22">
   <si>
     <t>REPORTE POR EMPRESA</t>
   </si>
@@ -26,7 +26,7 @@
     <t>T.T.</t>
   </si>
   <si>
-    <t>$800m.n.</t>
+    <t>$400m.n.</t>
   </si>
   <si>
     <t># Ticket</t>
@@ -56,34 +56,31 @@
     <t>Punto venta</t>
   </si>
   <si>
+    <t>Tipo de pago</t>
+  </si>
+  <si>
     <t>NO</t>
   </si>
   <si>
     <t>Modulo 5</t>
   </si>
   <si>
-    <t>Bandera</t>
+    <t>Efectivo</t>
   </si>
   <si>
-    <t>2025-10-01 08:17:33</t>
+    <t>2026-02-13 10:51:26</t>
   </si>
   <si>
-    <t>g.otay</t>
+    <t xml:space="preserve">recomendar hotel </t>
   </si>
   <si>
     <t>ivan</t>
   </si>
   <si>
-    <t>Fernando</t>
+    <t>victor</t>
   </si>
   <si>
     <t>$400</t>
-  </si>
-  <si>
-    <t>2025-10-01 08:17:41</t>
-  </si>
-  <si>
-    <t xml:space="preserve">san isidro </t>
   </si>
 </sst>
 </file>
@@ -94,7 +91,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0;[Red]\-&quot;$&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00;[Red]\-&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -110,7 +107,7 @@
       <strike val="0"/>
       <u val="none"/>
       <sz val="24"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -119,7 +116,7 @@
       <strike val="0"/>
       <u val="none"/>
       <sz val="18"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -145,7 +142,25 @@
       <i val="0"/>
       <strike val="0"/>
       <u val="none"/>
+      <sz val="24"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="18"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
@@ -159,7 +174,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF000000"/>
+        <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
@@ -176,7 +191,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
@@ -188,13 +203,12 @@
     <xf xfId="0" fontId="4" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="4" numFmtId="164" fillId="0" borderId="0" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="4" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="6" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="0" numFmtId="165" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="2" numFmtId="164" fillId="0" borderId="0" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="4" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="7" numFmtId="164" fillId="0" borderId="0" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="0" numFmtId="165" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -507,6 +521,7 @@
     <col min="7" max="7" width="16.571428571429" customWidth="true" style="0"/>
     <col min="8" max="8" width="14.428571428571" customWidth="true" style="0"/>
     <col min="9" max="9" width="16.714285714286" customWidth="true" style="0"/>
+    <col min="10" max="10" width="16.285714285714" customWidth="true" style="0"/>
     <col min="14" max="14" width="17.714285714286" customWidth="true" style="0"/>
     <col min="15" max="15" width="22.571428571429" customWidth="true" style="0"/>
     <col min="16" max="16" width="15.285714285714" customWidth="true" style="0"/>
@@ -633,36 +648,41 @@
       <c r="I7" s="3" t="s">
         <v>12</v>
       </c>
+      <c r="J7" s="3" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="8" spans="1:17">
       <c r="A8">
-        <v>337302</v>
+        <v>337323</v>
       </c>
       <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8">
+        <v>2</v>
+      </c>
+      <c r="G8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J8" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" t="s">
-        <v>19</v>
-      </c>
-      <c r="F8">
-        <v>1</v>
-      </c>
-      <c r="G8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
       <c r="N8" s="8"/>
@@ -671,33 +691,8 @@
       <c r="Q8" s="8"/>
     </row>
     <row r="9" spans="1:17">
-      <c r="A9">
-        <v>337303</v>
-      </c>
-      <c r="B9" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" t="s">
-        <v>18</v>
-      </c>
-      <c r="E9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9">
-        <v>1</v>
-      </c>
-      <c r="G9" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
       <c r="J9" s="7"/>
       <c r="K9" s="7"/>
       <c r="L9" s="7"/>
@@ -747,7 +742,7 @@
       <c r="L13" s="7"/>
       <c r="O13" s="10"/>
       <c r="P13" s="11"/>
-      <c r="Q13" s="14"/>
+      <c r="Q13" s="13"/>
     </row>
     <row r="14" spans="1:17" customHeight="1" ht="23.25">
       <c r="H14" s="5"/>
@@ -758,7 +753,7 @@
     </row>
     <row r="15" spans="1:17" customHeight="1" ht="15.75">
       <c r="H15" s="6"/>
-      <c r="I15" s="13"/>
+      <c r="I15" s="6"/>
     </row>
     <row r="16" spans="1:17" customHeight="1" ht="31.5">
       <c r="H16" s="4"/>
@@ -833,1782 +828,1782 @@
     </row>
     <row r="23" spans="1:17" customHeight="1" ht="15.75">
       <c r="H23" s="6"/>
-      <c r="I23" s="13"/>
+      <c r="I23" s="6"/>
     </row>
     <row r="24" spans="1:17" customHeight="1" ht="15.75">
       <c r="H24" s="6"/>
-      <c r="I24" s="13"/>
+      <c r="I24" s="6"/>
     </row>
     <row r="25" spans="1:17" customHeight="1" ht="15.75">
       <c r="H25" s="6"/>
-      <c r="I25" s="13"/>
+      <c r="I25" s="6"/>
     </row>
     <row r="26" spans="1:17" customHeight="1" ht="15.75">
       <c r="H26" s="6"/>
-      <c r="I26" s="13"/>
+      <c r="I26" s="6"/>
     </row>
     <row r="27" spans="1:17" customHeight="1" ht="15.75">
       <c r="H27" s="6"/>
-      <c r="I27" s="13"/>
+      <c r="I27" s="6"/>
     </row>
     <row r="28" spans="1:17" customHeight="1" ht="15.75">
       <c r="H28" s="6"/>
-      <c r="I28" s="13"/>
+      <c r="I28" s="6"/>
     </row>
     <row r="29" spans="1:17" customHeight="1" ht="15.75">
       <c r="H29" s="6"/>
-      <c r="I29" s="13"/>
+      <c r="I29" s="6"/>
     </row>
     <row r="30" spans="1:17" customHeight="1" ht="15.75">
       <c r="H30" s="6"/>
-      <c r="I30" s="13"/>
+      <c r="I30" s="6"/>
     </row>
     <row r="31" spans="1:17" customHeight="1" ht="15.75">
       <c r="H31" s="6"/>
-      <c r="I31" s="13"/>
+      <c r="I31" s="6"/>
     </row>
     <row r="32" spans="1:17" customHeight="1" ht="15.75">
       <c r="H32" s="6"/>
-      <c r="I32" s="13"/>
+      <c r="I32" s="6"/>
     </row>
     <row r="33" spans="1:17" customHeight="1" ht="15.75">
       <c r="H33" s="6"/>
-      <c r="I33" s="13"/>
+      <c r="I33" s="6"/>
     </row>
     <row r="34" spans="1:17" customHeight="1" ht="15.75">
       <c r="H34" s="6"/>
-      <c r="I34" s="13"/>
+      <c r="I34" s="6"/>
     </row>
     <row r="35" spans="1:17" customHeight="1" ht="15.75">
       <c r="H35" s="6"/>
-      <c r="I35" s="13"/>
+      <c r="I35" s="6"/>
     </row>
     <row r="36" spans="1:17" customHeight="1" ht="15.75">
       <c r="H36" s="6"/>
-      <c r="I36" s="13"/>
+      <c r="I36" s="6"/>
     </row>
     <row r="37" spans="1:17" customHeight="1" ht="15.75">
       <c r="H37" s="6"/>
-      <c r="I37" s="13"/>
+      <c r="I37" s="6"/>
     </row>
     <row r="38" spans="1:17" customHeight="1" ht="15.75">
       <c r="H38" s="6"/>
-      <c r="I38" s="13"/>
+      <c r="I38" s="6"/>
     </row>
     <row r="39" spans="1:17" customHeight="1" ht="15.75">
       <c r="H39" s="6"/>
-      <c r="I39" s="13"/>
+      <c r="I39" s="6"/>
     </row>
     <row r="40" spans="1:17" customHeight="1" ht="15.75">
       <c r="H40" s="6"/>
-      <c r="I40" s="13"/>
+      <c r="I40" s="6"/>
     </row>
     <row r="41" spans="1:17" customHeight="1" ht="15.75">
       <c r="H41" s="6"/>
-      <c r="I41" s="13"/>
+      <c r="I41" s="6"/>
     </row>
     <row r="42" spans="1:17" customHeight="1" ht="15.75">
       <c r="H42" s="6"/>
-      <c r="I42" s="13"/>
+      <c r="I42" s="6"/>
     </row>
     <row r="43" spans="1:17" customHeight="1" ht="15.75">
       <c r="H43" s="6"/>
-      <c r="I43" s="13"/>
+      <c r="I43" s="6"/>
     </row>
     <row r="44" spans="1:17" customHeight="1" ht="15.75">
       <c r="H44" s="6"/>
-      <c r="I44" s="13"/>
+      <c r="I44" s="6"/>
     </row>
     <row r="45" spans="1:17" customHeight="1" ht="15.75">
       <c r="H45" s="6"/>
-      <c r="I45" s="13"/>
+      <c r="I45" s="6"/>
     </row>
     <row r="46" spans="1:17" customHeight="1" ht="15.75">
       <c r="H46" s="6"/>
-      <c r="I46" s="13"/>
+      <c r="I46" s="6"/>
     </row>
     <row r="47" spans="1:17" customHeight="1" ht="15.75">
       <c r="H47" s="6"/>
-      <c r="I47" s="13"/>
+      <c r="I47" s="6"/>
     </row>
     <row r="48" spans="1:17" customHeight="1" ht="15.75">
       <c r="H48" s="6"/>
-      <c r="I48" s="13"/>
+      <c r="I48" s="6"/>
     </row>
     <row r="49" spans="1:17" customHeight="1" ht="15.75">
       <c r="H49" s="6"/>
-      <c r="I49" s="13"/>
+      <c r="I49" s="6"/>
     </row>
     <row r="50" spans="1:17" customHeight="1" ht="15.75">
       <c r="H50" s="6"/>
-      <c r="I50" s="13"/>
+      <c r="I50" s="6"/>
     </row>
     <row r="51" spans="1:17" customHeight="1" ht="15.75">
       <c r="H51" s="6"/>
-      <c r="I51" s="13"/>
+      <c r="I51" s="6"/>
     </row>
     <row r="52" spans="1:17" customHeight="1" ht="15.75">
       <c r="H52" s="6"/>
-      <c r="I52" s="13"/>
+      <c r="I52" s="6"/>
     </row>
     <row r="53" spans="1:17" customHeight="1" ht="15.75">
       <c r="H53" s="6"/>
-      <c r="I53" s="13"/>
+      <c r="I53" s="6"/>
     </row>
     <row r="54" spans="1:17" customHeight="1" ht="15.75">
       <c r="H54" s="6"/>
-      <c r="I54" s="13"/>
+      <c r="I54" s="6"/>
     </row>
     <row r="55" spans="1:17" customHeight="1" ht="15.75">
       <c r="H55" s="6"/>
-      <c r="I55" s="13"/>
+      <c r="I55" s="6"/>
     </row>
     <row r="56" spans="1:17" customHeight="1" ht="15.75">
       <c r="H56" s="6"/>
-      <c r="I56" s="13"/>
+      <c r="I56" s="6"/>
     </row>
     <row r="57" spans="1:17" customHeight="1" ht="15.75">
       <c r="H57" s="6"/>
-      <c r="I57" s="13"/>
+      <c r="I57" s="6"/>
     </row>
     <row r="58" spans="1:17" customHeight="1" ht="15.75">
       <c r="H58" s="6"/>
-      <c r="I58" s="13"/>
+      <c r="I58" s="6"/>
     </row>
     <row r="59" spans="1:17" customHeight="1" ht="15.75">
       <c r="H59" s="6"/>
-      <c r="I59" s="13"/>
+      <c r="I59" s="6"/>
     </row>
     <row r="60" spans="1:17" customHeight="1" ht="15.75">
       <c r="H60" s="6"/>
-      <c r="I60" s="13"/>
+      <c r="I60" s="6"/>
     </row>
     <row r="61" spans="1:17" customHeight="1" ht="15.75">
       <c r="H61" s="6"/>
-      <c r="I61" s="13"/>
+      <c r="I61" s="6"/>
     </row>
     <row r="62" spans="1:17" customHeight="1" ht="15.75">
       <c r="H62" s="6"/>
-      <c r="I62" s="13"/>
+      <c r="I62" s="6"/>
     </row>
     <row r="63" spans="1:17" customHeight="1" ht="15.75">
       <c r="H63" s="6"/>
-      <c r="I63" s="13"/>
+      <c r="I63" s="6"/>
     </row>
     <row r="64" spans="1:17" customHeight="1" ht="15.75">
       <c r="H64" s="6"/>
-      <c r="I64" s="13"/>
+      <c r="I64" s="6"/>
     </row>
     <row r="65" spans="1:17" customHeight="1" ht="15.75">
       <c r="H65" s="6"/>
-      <c r="I65" s="13"/>
+      <c r="I65" s="6"/>
     </row>
     <row r="66" spans="1:17" customHeight="1" ht="15.75">
       <c r="H66" s="6"/>
-      <c r="I66" s="13"/>
+      <c r="I66" s="6"/>
     </row>
     <row r="67" spans="1:17" customHeight="1" ht="15.75">
       <c r="H67" s="6"/>
-      <c r="I67" s="13"/>
+      <c r="I67" s="6"/>
     </row>
     <row r="68" spans="1:17" customHeight="1" ht="15.75">
       <c r="H68" s="6"/>
-      <c r="I68" s="13"/>
+      <c r="I68" s="6"/>
     </row>
     <row r="69" spans="1:17" customHeight="1" ht="15.75">
       <c r="H69" s="6"/>
-      <c r="I69" s="13"/>
+      <c r="I69" s="6"/>
     </row>
     <row r="70" spans="1:17" customHeight="1" ht="15.75">
       <c r="H70" s="6"/>
-      <c r="I70" s="13"/>
+      <c r="I70" s="6"/>
     </row>
     <row r="71" spans="1:17" customHeight="1" ht="15.75">
       <c r="H71" s="6"/>
-      <c r="I71" s="13"/>
+      <c r="I71" s="6"/>
     </row>
     <row r="72" spans="1:17" customHeight="1" ht="15.75">
       <c r="H72" s="6"/>
-      <c r="I72" s="13"/>
+      <c r="I72" s="6"/>
     </row>
     <row r="73" spans="1:17" customHeight="1" ht="15.75">
       <c r="H73" s="6"/>
-      <c r="I73" s="13"/>
+      <c r="I73" s="6"/>
     </row>
     <row r="74" spans="1:17" customHeight="1" ht="15.75">
       <c r="H74" s="6"/>
-      <c r="I74" s="13"/>
+      <c r="I74" s="6"/>
     </row>
     <row r="75" spans="1:17" customHeight="1" ht="15.75">
       <c r="H75" s="6"/>
-      <c r="I75" s="13"/>
+      <c r="I75" s="6"/>
     </row>
     <row r="76" spans="1:17" customHeight="1" ht="15.75">
       <c r="H76" s="6"/>
-      <c r="I76" s="13"/>
+      <c r="I76" s="6"/>
     </row>
     <row r="77" spans="1:17" customHeight="1" ht="15.75">
       <c r="H77" s="6"/>
-      <c r="I77" s="13"/>
+      <c r="I77" s="6"/>
     </row>
     <row r="78" spans="1:17" customHeight="1" ht="15.75">
       <c r="H78" s="6"/>
-      <c r="I78" s="13"/>
+      <c r="I78" s="6"/>
     </row>
     <row r="79" spans="1:17" customHeight="1" ht="15.75">
       <c r="H79" s="6"/>
-      <c r="I79" s="13"/>
+      <c r="I79" s="6"/>
     </row>
     <row r="80" spans="1:17" customHeight="1" ht="15.75">
       <c r="H80" s="6"/>
-      <c r="I80" s="13"/>
+      <c r="I80" s="6"/>
     </row>
     <row r="81" spans="1:17" customHeight="1" ht="15.75">
       <c r="H81" s="6"/>
-      <c r="I81" s="13"/>
+      <c r="I81" s="6"/>
     </row>
     <row r="82" spans="1:17" customHeight="1" ht="15.75">
       <c r="H82" s="6"/>
-      <c r="I82" s="13"/>
+      <c r="I82" s="6"/>
     </row>
     <row r="83" spans="1:17" customHeight="1" ht="15.75">
       <c r="H83" s="6"/>
-      <c r="I83" s="13"/>
+      <c r="I83" s="6"/>
     </row>
     <row r="84" spans="1:17" customHeight="1" ht="15.75">
       <c r="H84" s="6"/>
-      <c r="I84" s="13"/>
+      <c r="I84" s="6"/>
     </row>
     <row r="85" spans="1:17" customHeight="1" ht="15.75">
       <c r="H85" s="6"/>
-      <c r="I85" s="13"/>
+      <c r="I85" s="6"/>
     </row>
     <row r="86" spans="1:17" customHeight="1" ht="15.75">
       <c r="H86" s="6"/>
-      <c r="I86" s="13"/>
+      <c r="I86" s="6"/>
     </row>
     <row r="87" spans="1:17" customHeight="1" ht="15.75">
       <c r="H87" s="6"/>
-      <c r="I87" s="13"/>
+      <c r="I87" s="6"/>
     </row>
     <row r="88" spans="1:17" customHeight="1" ht="15.75">
       <c r="H88" s="6"/>
-      <c r="I88" s="13"/>
+      <c r="I88" s="6"/>
     </row>
     <row r="89" spans="1:17" customHeight="1" ht="15.75">
       <c r="H89" s="6"/>
-      <c r="I89" s="13"/>
+      <c r="I89" s="6"/>
     </row>
     <row r="90" spans="1:17" customHeight="1" ht="15.75">
       <c r="H90" s="6"/>
-      <c r="I90" s="13"/>
+      <c r="I90" s="6"/>
     </row>
     <row r="91" spans="1:17" customHeight="1" ht="15.75">
       <c r="H91" s="6"/>
-      <c r="I91" s="13"/>
+      <c r="I91" s="6"/>
     </row>
     <row r="92" spans="1:17" customHeight="1" ht="15.75">
       <c r="H92" s="6"/>
-      <c r="I92" s="13"/>
+      <c r="I92" s="6"/>
     </row>
     <row r="93" spans="1:17" customHeight="1" ht="15.75">
       <c r="H93" s="6"/>
-      <c r="I93" s="13"/>
+      <c r="I93" s="6"/>
     </row>
     <row r="94" spans="1:17" customHeight="1" ht="15.75">
       <c r="H94" s="6"/>
-      <c r="I94" s="13"/>
+      <c r="I94" s="6"/>
     </row>
     <row r="95" spans="1:17" customHeight="1" ht="15.75">
       <c r="H95" s="6"/>
-      <c r="I95" s="13"/>
+      <c r="I95" s="6"/>
     </row>
     <row r="96" spans="1:17" customHeight="1" ht="15.75">
       <c r="H96" s="6"/>
-      <c r="I96" s="13"/>
+      <c r="I96" s="6"/>
     </row>
     <row r="97" spans="1:17" customHeight="1" ht="15.75">
       <c r="H97" s="6"/>
-      <c r="I97" s="13"/>
+      <c r="I97" s="6"/>
     </row>
     <row r="98" spans="1:17" customHeight="1" ht="15.75">
       <c r="H98" s="6"/>
-      <c r="I98" s="13"/>
+      <c r="I98" s="6"/>
     </row>
     <row r="99" spans="1:17" customHeight="1" ht="15.75">
       <c r="H99" s="6"/>
-      <c r="I99" s="13"/>
+      <c r="I99" s="6"/>
     </row>
     <row r="100" spans="1:17" customHeight="1" ht="15.75">
       <c r="H100" s="6"/>
-      <c r="I100" s="13"/>
+      <c r="I100" s="6"/>
     </row>
     <row r="101" spans="1:17" customHeight="1" ht="15.75">
       <c r="H101" s="6"/>
-      <c r="I101" s="13"/>
+      <c r="I101" s="6"/>
     </row>
     <row r="102" spans="1:17" customHeight="1" ht="15.75">
       <c r="H102" s="6"/>
-      <c r="I102" s="13"/>
+      <c r="I102" s="6"/>
     </row>
     <row r="103" spans="1:17" customHeight="1" ht="15.75">
       <c r="H103" s="6"/>
-      <c r="I103" s="13"/>
+      <c r="I103" s="6"/>
     </row>
     <row r="104" spans="1:17" customHeight="1" ht="15.75">
       <c r="H104" s="6"/>
-      <c r="I104" s="13"/>
+      <c r="I104" s="6"/>
     </row>
     <row r="105" spans="1:17" customHeight="1" ht="15.75">
       <c r="H105" s="6"/>
-      <c r="I105" s="13"/>
+      <c r="I105" s="6"/>
     </row>
     <row r="106" spans="1:17" customHeight="1" ht="15.75">
       <c r="H106" s="6"/>
-      <c r="I106" s="13"/>
+      <c r="I106" s="6"/>
     </row>
     <row r="107" spans="1:17" customHeight="1" ht="15.75">
       <c r="H107" s="6"/>
-      <c r="I107" s="13"/>
+      <c r="I107" s="6"/>
     </row>
     <row r="108" spans="1:17" customHeight="1" ht="15.75">
       <c r="H108" s="6"/>
-      <c r="I108" s="13"/>
+      <c r="I108" s="6"/>
     </row>
     <row r="109" spans="1:17" customHeight="1" ht="15.75">
       <c r="H109" s="6"/>
-      <c r="I109" s="13"/>
+      <c r="I109" s="6"/>
     </row>
     <row r="110" spans="1:17" customHeight="1" ht="15.75">
       <c r="H110" s="6"/>
-      <c r="I110" s="13"/>
+      <c r="I110" s="6"/>
     </row>
     <row r="111" spans="1:17" customHeight="1" ht="15.75">
       <c r="H111" s="6"/>
-      <c r="I111" s="13"/>
+      <c r="I111" s="6"/>
     </row>
     <row r="112" spans="1:17" customHeight="1" ht="15.75">
       <c r="H112" s="6"/>
-      <c r="I112" s="13"/>
+      <c r="I112" s="6"/>
     </row>
     <row r="113" spans="1:17" customHeight="1" ht="15.75">
       <c r="H113" s="6"/>
-      <c r="I113" s="13"/>
+      <c r="I113" s="6"/>
     </row>
     <row r="114" spans="1:17" customHeight="1" ht="15.75">
       <c r="H114" s="6"/>
-      <c r="I114" s="13"/>
+      <c r="I114" s="6"/>
     </row>
     <row r="115" spans="1:17" customHeight="1" ht="15.75">
       <c r="H115" s="6"/>
-      <c r="I115" s="13"/>
+      <c r="I115" s="6"/>
     </row>
     <row r="116" spans="1:17" customHeight="1" ht="15.75">
       <c r="H116" s="6"/>
-      <c r="I116" s="13"/>
+      <c r="I116" s="6"/>
     </row>
     <row r="117" spans="1:17" customHeight="1" ht="15.75">
       <c r="H117" s="6"/>
-      <c r="I117" s="13"/>
+      <c r="I117" s="6"/>
     </row>
     <row r="118" spans="1:17" customHeight="1" ht="15.75">
       <c r="H118" s="6"/>
-      <c r="I118" s="13"/>
+      <c r="I118" s="6"/>
     </row>
     <row r="119" spans="1:17" customHeight="1" ht="15.75">
       <c r="H119" s="6"/>
-      <c r="I119" s="13"/>
+      <c r="I119" s="6"/>
     </row>
     <row r="120" spans="1:17" customHeight="1" ht="15.75">
       <c r="H120" s="6"/>
-      <c r="I120" s="13"/>
+      <c r="I120" s="6"/>
     </row>
     <row r="121" spans="1:17" customHeight="1" ht="15.75">
       <c r="H121" s="6"/>
-      <c r="I121" s="13"/>
+      <c r="I121" s="6"/>
     </row>
     <row r="122" spans="1:17" customHeight="1" ht="15.75">
       <c r="H122" s="6"/>
-      <c r="I122" s="13"/>
+      <c r="I122" s="6"/>
     </row>
     <row r="123" spans="1:17" customHeight="1" ht="15.75">
       <c r="H123" s="6"/>
-      <c r="I123" s="13"/>
+      <c r="I123" s="6"/>
     </row>
     <row r="124" spans="1:17" customHeight="1" ht="15.75">
       <c r="H124" s="6"/>
-      <c r="I124" s="13"/>
+      <c r="I124" s="6"/>
     </row>
     <row r="125" spans="1:17" customHeight="1" ht="15.75">
       <c r="H125" s="6"/>
-      <c r="I125" s="13"/>
+      <c r="I125" s="6"/>
     </row>
     <row r="126" spans="1:17" customHeight="1" ht="15.75">
       <c r="H126" s="6"/>
-      <c r="I126" s="13"/>
+      <c r="I126" s="6"/>
     </row>
     <row r="127" spans="1:17" customHeight="1" ht="15.75">
       <c r="H127" s="6"/>
-      <c r="I127" s="13"/>
+      <c r="I127" s="6"/>
     </row>
     <row r="128" spans="1:17" customHeight="1" ht="15.75">
       <c r="H128" s="6"/>
-      <c r="I128" s="13"/>
+      <c r="I128" s="6"/>
     </row>
     <row r="129" spans="1:17" customHeight="1" ht="15.75">
       <c r="H129" s="6"/>
-      <c r="I129" s="13"/>
+      <c r="I129" s="6"/>
     </row>
     <row r="130" spans="1:17" customHeight="1" ht="15.75">
       <c r="H130" s="6"/>
-      <c r="I130" s="13"/>
+      <c r="I130" s="6"/>
     </row>
     <row r="131" spans="1:17" customHeight="1" ht="15.75">
       <c r="H131" s="6"/>
-      <c r="I131" s="13"/>
+      <c r="I131" s="6"/>
     </row>
     <row r="132" spans="1:17" customHeight="1" ht="15.75">
       <c r="H132" s="6"/>
-      <c r="I132" s="13"/>
+      <c r="I132" s="6"/>
     </row>
     <row r="133" spans="1:17" customHeight="1" ht="15.75">
       <c r="H133" s="6"/>
-      <c r="I133" s="13"/>
+      <c r="I133" s="6"/>
     </row>
     <row r="134" spans="1:17" customHeight="1" ht="15.75">
       <c r="H134" s="6"/>
-      <c r="I134" s="13"/>
+      <c r="I134" s="6"/>
     </row>
     <row r="135" spans="1:17" customHeight="1" ht="15.75">
       <c r="H135" s="6"/>
-      <c r="I135" s="13"/>
+      <c r="I135" s="6"/>
     </row>
     <row r="136" spans="1:17" customHeight="1" ht="15.75">
       <c r="H136" s="6"/>
-      <c r="I136" s="13"/>
+      <c r="I136" s="6"/>
     </row>
     <row r="137" spans="1:17" customHeight="1" ht="15.75">
       <c r="H137" s="6"/>
-      <c r="I137" s="13"/>
+      <c r="I137" s="6"/>
     </row>
     <row r="138" spans="1:17" customHeight="1" ht="15.75">
       <c r="H138" s="6"/>
-      <c r="I138" s="13"/>
+      <c r="I138" s="6"/>
     </row>
     <row r="139" spans="1:17" customHeight="1" ht="15.75">
       <c r="H139" s="6"/>
-      <c r="I139" s="13"/>
+      <c r="I139" s="6"/>
     </row>
     <row r="140" spans="1:17" customHeight="1" ht="15.75">
       <c r="H140" s="6"/>
-      <c r="I140" s="13"/>
+      <c r="I140" s="6"/>
     </row>
     <row r="141" spans="1:17" customHeight="1" ht="15.75">
       <c r="H141" s="6"/>
-      <c r="I141" s="13"/>
+      <c r="I141" s="6"/>
     </row>
     <row r="142" spans="1:17" customHeight="1" ht="15.75">
       <c r="H142" s="6"/>
-      <c r="I142" s="13"/>
+      <c r="I142" s="6"/>
     </row>
     <row r="143" spans="1:17" customHeight="1" ht="15.75">
       <c r="H143" s="6"/>
-      <c r="I143" s="13"/>
+      <c r="I143" s="6"/>
     </row>
     <row r="144" spans="1:17" customHeight="1" ht="15.75">
       <c r="H144" s="6"/>
-      <c r="I144" s="13"/>
+      <c r="I144" s="6"/>
     </row>
     <row r="145" spans="1:17" customHeight="1" ht="15.75">
       <c r="H145" s="6"/>
-      <c r="I145" s="13"/>
+      <c r="I145" s="6"/>
     </row>
     <row r="146" spans="1:17" customHeight="1" ht="15.75">
       <c r="H146" s="6"/>
-      <c r="I146" s="13"/>
+      <c r="I146" s="6"/>
     </row>
     <row r="147" spans="1:17" customHeight="1" ht="15.75">
       <c r="H147" s="6"/>
-      <c r="I147" s="13"/>
+      <c r="I147" s="6"/>
     </row>
     <row r="148" spans="1:17" customHeight="1" ht="15.75">
       <c r="H148" s="6"/>
-      <c r="I148" s="13"/>
+      <c r="I148" s="6"/>
     </row>
     <row r="149" spans="1:17" customHeight="1" ht="15.75">
       <c r="H149" s="6"/>
-      <c r="I149" s="13"/>
+      <c r="I149" s="6"/>
     </row>
     <row r="150" spans="1:17" customHeight="1" ht="15.75">
       <c r="H150" s="6"/>
-      <c r="I150" s="13"/>
+      <c r="I150" s="6"/>
     </row>
     <row r="151" spans="1:17" customHeight="1" ht="15.75">
       <c r="H151" s="6"/>
-      <c r="I151" s="13"/>
+      <c r="I151" s="6"/>
     </row>
     <row r="152" spans="1:17" customHeight="1" ht="15.75">
       <c r="H152" s="6"/>
-      <c r="I152" s="13"/>
+      <c r="I152" s="6"/>
     </row>
     <row r="153" spans="1:17" customHeight="1" ht="15.75">
       <c r="H153" s="6"/>
-      <c r="I153" s="13"/>
+      <c r="I153" s="6"/>
     </row>
     <row r="154" spans="1:17" customHeight="1" ht="15.75">
       <c r="H154" s="6"/>
-      <c r="I154" s="13"/>
+      <c r="I154" s="6"/>
     </row>
     <row r="155" spans="1:17" customHeight="1" ht="15.75">
       <c r="H155" s="6"/>
-      <c r="I155" s="13"/>
+      <c r="I155" s="6"/>
     </row>
     <row r="156" spans="1:17" customHeight="1" ht="15.75">
       <c r="H156" s="6"/>
-      <c r="I156" s="13"/>
+      <c r="I156" s="6"/>
     </row>
     <row r="157" spans="1:17" customHeight="1" ht="15.75">
       <c r="H157" s="6"/>
-      <c r="I157" s="13"/>
+      <c r="I157" s="6"/>
     </row>
     <row r="158" spans="1:17" customHeight="1" ht="15.75">
       <c r="H158" s="6"/>
-      <c r="I158" s="13"/>
+      <c r="I158" s="6"/>
     </row>
     <row r="159" spans="1:17" customHeight="1" ht="15.75">
       <c r="H159" s="6"/>
-      <c r="I159" s="13"/>
+      <c r="I159" s="6"/>
     </row>
     <row r="160" spans="1:17" customHeight="1" ht="15.75">
       <c r="H160" s="6"/>
-      <c r="I160" s="13"/>
+      <c r="I160" s="6"/>
     </row>
     <row r="161" spans="1:17" customHeight="1" ht="15.75">
       <c r="H161" s="6"/>
-      <c r="I161" s="13"/>
+      <c r="I161" s="6"/>
     </row>
     <row r="162" spans="1:17" customHeight="1" ht="15.75">
       <c r="H162" s="6"/>
-      <c r="I162" s="13"/>
+      <c r="I162" s="6"/>
     </row>
     <row r="163" spans="1:17" customHeight="1" ht="15.75">
       <c r="H163" s="6"/>
-      <c r="I163" s="13"/>
+      <c r="I163" s="6"/>
     </row>
     <row r="164" spans="1:17" customHeight="1" ht="15.75">
       <c r="H164" s="6"/>
-      <c r="I164" s="13"/>
+      <c r="I164" s="6"/>
     </row>
     <row r="165" spans="1:17" customHeight="1" ht="15.75">
       <c r="H165" s="6"/>
-      <c r="I165" s="13"/>
+      <c r="I165" s="6"/>
     </row>
     <row r="166" spans="1:17" customHeight="1" ht="15.75">
       <c r="H166" s="6"/>
-      <c r="I166" s="13"/>
+      <c r="I166" s="6"/>
     </row>
     <row r="167" spans="1:17" customHeight="1" ht="15.75">
       <c r="H167" s="6"/>
-      <c r="I167" s="13"/>
+      <c r="I167" s="6"/>
     </row>
     <row r="168" spans="1:17" customHeight="1" ht="15.75">
       <c r="H168" s="6"/>
-      <c r="I168" s="13"/>
+      <c r="I168" s="6"/>
     </row>
     <row r="169" spans="1:17" customHeight="1" ht="15.75">
       <c r="H169" s="6"/>
-      <c r="I169" s="13"/>
+      <c r="I169" s="6"/>
     </row>
     <row r="170" spans="1:17" customHeight="1" ht="15.75">
       <c r="H170" s="6"/>
-      <c r="I170" s="13"/>
+      <c r="I170" s="6"/>
     </row>
     <row r="171" spans="1:17" customHeight="1" ht="15.75">
       <c r="H171" s="6"/>
-      <c r="I171" s="13"/>
+      <c r="I171" s="6"/>
     </row>
     <row r="172" spans="1:17" customHeight="1" ht="15.75">
       <c r="H172" s="6"/>
-      <c r="I172" s="13"/>
+      <c r="I172" s="6"/>
     </row>
     <row r="173" spans="1:17" customHeight="1" ht="15.75">
       <c r="H173" s="6"/>
-      <c r="I173" s="13"/>
+      <c r="I173" s="6"/>
     </row>
     <row r="174" spans="1:17" customHeight="1" ht="15.75">
       <c r="H174" s="6"/>
-      <c r="I174" s="13"/>
+      <c r="I174" s="6"/>
     </row>
     <row r="175" spans="1:17" customHeight="1" ht="15.75">
       <c r="H175" s="6"/>
-      <c r="I175" s="13"/>
+      <c r="I175" s="6"/>
     </row>
     <row r="176" spans="1:17" customHeight="1" ht="15.75">
       <c r="H176" s="6"/>
-      <c r="I176" s="13"/>
+      <c r="I176" s="6"/>
     </row>
     <row r="177" spans="1:17" customHeight="1" ht="15.75">
       <c r="H177" s="6"/>
-      <c r="I177" s="13"/>
+      <c r="I177" s="6"/>
     </row>
     <row r="178" spans="1:17" customHeight="1" ht="15.75">
       <c r="H178" s="6"/>
-      <c r="I178" s="13"/>
+      <c r="I178" s="6"/>
     </row>
     <row r="179" spans="1:17" customHeight="1" ht="15.75">
       <c r="H179" s="6"/>
-      <c r="I179" s="13"/>
+      <c r="I179" s="6"/>
     </row>
     <row r="180" spans="1:17" customHeight="1" ht="15.75">
       <c r="H180" s="6"/>
-      <c r="I180" s="13"/>
+      <c r="I180" s="6"/>
     </row>
     <row r="181" spans="1:17" customHeight="1" ht="15.75">
       <c r="H181" s="6"/>
-      <c r="I181" s="13"/>
+      <c r="I181" s="6"/>
     </row>
     <row r="182" spans="1:17" customHeight="1" ht="15.75">
       <c r="H182" s="6"/>
-      <c r="I182" s="13"/>
+      <c r="I182" s="6"/>
     </row>
     <row r="183" spans="1:17" customHeight="1" ht="15.75">
       <c r="H183" s="6"/>
-      <c r="I183" s="13"/>
+      <c r="I183" s="6"/>
     </row>
     <row r="184" spans="1:17" customHeight="1" ht="15.75">
       <c r="H184" s="6"/>
-      <c r="I184" s="13"/>
+      <c r="I184" s="6"/>
     </row>
     <row r="185" spans="1:17" customHeight="1" ht="15.75">
       <c r="H185" s="6"/>
-      <c r="I185" s="13"/>
+      <c r="I185" s="6"/>
     </row>
     <row r="186" spans="1:17" customHeight="1" ht="15.75">
       <c r="H186" s="6"/>
-      <c r="I186" s="13"/>
+      <c r="I186" s="6"/>
     </row>
     <row r="187" spans="1:17" customHeight="1" ht="15.75">
       <c r="H187" s="6"/>
-      <c r="I187" s="13"/>
+      <c r="I187" s="6"/>
     </row>
     <row r="188" spans="1:17" customHeight="1" ht="15.75">
       <c r="H188" s="6"/>
-      <c r="I188" s="13"/>
+      <c r="I188" s="6"/>
     </row>
     <row r="189" spans="1:17" customHeight="1" ht="15.75">
       <c r="H189" s="6"/>
-      <c r="I189" s="13"/>
+      <c r="I189" s="6"/>
     </row>
     <row r="190" spans="1:17" customHeight="1" ht="15.75">
       <c r="H190" s="6"/>
-      <c r="I190" s="13"/>
+      <c r="I190" s="6"/>
     </row>
     <row r="191" spans="1:17" customHeight="1" ht="15.75">
       <c r="H191" s="6"/>
-      <c r="I191" s="13"/>
+      <c r="I191" s="6"/>
     </row>
     <row r="192" spans="1:17" customHeight="1" ht="15.75">
       <c r="H192" s="6"/>
-      <c r="I192" s="13"/>
+      <c r="I192" s="6"/>
     </row>
     <row r="193" spans="1:17" customHeight="1" ht="15.75">
       <c r="H193" s="6"/>
-      <c r="I193" s="13"/>
+      <c r="I193" s="6"/>
     </row>
     <row r="194" spans="1:17" customHeight="1" ht="15.75">
       <c r="H194" s="6"/>
-      <c r="I194" s="13"/>
+      <c r="I194" s="6"/>
     </row>
     <row r="195" spans="1:17" customHeight="1" ht="15.75">
       <c r="H195" s="6"/>
-      <c r="I195" s="13"/>
+      <c r="I195" s="6"/>
     </row>
     <row r="196" spans="1:17" customHeight="1" ht="15.75">
       <c r="H196" s="6"/>
-      <c r="I196" s="13"/>
+      <c r="I196" s="6"/>
     </row>
     <row r="197" spans="1:17" customHeight="1" ht="15.75">
       <c r="H197" s="6"/>
-      <c r="I197" s="13"/>
+      <c r="I197" s="6"/>
     </row>
     <row r="198" spans="1:17" customHeight="1" ht="15.75">
       <c r="H198" s="6"/>
-      <c r="I198" s="13"/>
+      <c r="I198" s="6"/>
     </row>
     <row r="199" spans="1:17" customHeight="1" ht="15.75">
       <c r="H199" s="6"/>
-      <c r="I199" s="13"/>
+      <c r="I199" s="6"/>
     </row>
     <row r="200" spans="1:17" customHeight="1" ht="15.75">
       <c r="H200" s="6"/>
-      <c r="I200" s="13"/>
+      <c r="I200" s="6"/>
     </row>
     <row r="201" spans="1:17" customHeight="1" ht="15.75">
       <c r="H201" s="6"/>
-      <c r="I201" s="13"/>
+      <c r="I201" s="6"/>
     </row>
     <row r="202" spans="1:17" customHeight="1" ht="15.75">
       <c r="H202" s="6"/>
-      <c r="I202" s="13"/>
+      <c r="I202" s="6"/>
     </row>
     <row r="203" spans="1:17" customHeight="1" ht="15.75">
       <c r="H203" s="6"/>
-      <c r="I203" s="13"/>
+      <c r="I203" s="6"/>
     </row>
     <row r="204" spans="1:17" customHeight="1" ht="15.75">
       <c r="H204" s="6"/>
-      <c r="I204" s="13"/>
+      <c r="I204" s="6"/>
     </row>
     <row r="205" spans="1:17" customHeight="1" ht="15.75">
       <c r="H205" s="6"/>
-      <c r="I205" s="13"/>
+      <c r="I205" s="6"/>
     </row>
     <row r="206" spans="1:17" customHeight="1" ht="15.75">
       <c r="H206" s="6"/>
-      <c r="I206" s="13"/>
+      <c r="I206" s="6"/>
     </row>
     <row r="207" spans="1:17" customHeight="1" ht="15.75">
       <c r="H207" s="6"/>
-      <c r="I207" s="13"/>
+      <c r="I207" s="6"/>
     </row>
     <row r="208" spans="1:17" customHeight="1" ht="15.75">
       <c r="H208" s="6"/>
-      <c r="I208" s="13"/>
+      <c r="I208" s="6"/>
     </row>
     <row r="209" spans="1:17" customHeight="1" ht="15.75">
       <c r="H209" s="6"/>
-      <c r="I209" s="13"/>
+      <c r="I209" s="6"/>
     </row>
     <row r="210" spans="1:17" customHeight="1" ht="15.75">
       <c r="H210" s="6"/>
-      <c r="I210" s="13"/>
+      <c r="I210" s="6"/>
     </row>
     <row r="211" spans="1:17" customHeight="1" ht="15.75">
       <c r="H211" s="6"/>
-      <c r="I211" s="13"/>
+      <c r="I211" s="6"/>
     </row>
     <row r="212" spans="1:17" customHeight="1" ht="15.75">
       <c r="H212" s="6"/>
-      <c r="I212" s="13"/>
+      <c r="I212" s="6"/>
     </row>
     <row r="213" spans="1:17" customHeight="1" ht="15.75">
       <c r="H213" s="6"/>
-      <c r="I213" s="13"/>
+      <c r="I213" s="6"/>
     </row>
     <row r="214" spans="1:17" customHeight="1" ht="15.75">
       <c r="H214" s="6"/>
-      <c r="I214" s="13"/>
+      <c r="I214" s="6"/>
     </row>
     <row r="215" spans="1:17" customHeight="1" ht="15.75">
       <c r="H215" s="6"/>
-      <c r="I215" s="13"/>
+      <c r="I215" s="6"/>
     </row>
     <row r="216" spans="1:17" customHeight="1" ht="15.75">
       <c r="H216" s="6"/>
-      <c r="I216" s="13"/>
+      <c r="I216" s="6"/>
     </row>
     <row r="217" spans="1:17" customHeight="1" ht="15.75">
       <c r="H217" s="6"/>
-      <c r="I217" s="13"/>
+      <c r="I217" s="6"/>
     </row>
     <row r="218" spans="1:17" customHeight="1" ht="15.75">
       <c r="H218" s="6"/>
-      <c r="I218" s="13"/>
+      <c r="I218" s="6"/>
     </row>
     <row r="219" spans="1:17" customHeight="1" ht="15.75">
       <c r="H219" s="6"/>
-      <c r="I219" s="13"/>
+      <c r="I219" s="6"/>
     </row>
     <row r="220" spans="1:17" customHeight="1" ht="15.75">
       <c r="H220" s="6"/>
-      <c r="I220" s="13"/>
+      <c r="I220" s="6"/>
     </row>
     <row r="221" spans="1:17" customHeight="1" ht="15.75">
       <c r="H221" s="6"/>
-      <c r="I221" s="13"/>
+      <c r="I221" s="6"/>
     </row>
     <row r="222" spans="1:17" customHeight="1" ht="15.75">
       <c r="H222" s="6"/>
-      <c r="I222" s="13"/>
+      <c r="I222" s="6"/>
     </row>
     <row r="223" spans="1:17" customHeight="1" ht="15.75">
       <c r="H223" s="6"/>
-      <c r="I223" s="13"/>
+      <c r="I223" s="6"/>
     </row>
     <row r="224" spans="1:17" customHeight="1" ht="15.75">
       <c r="H224" s="6"/>
-      <c r="I224" s="13"/>
+      <c r="I224" s="6"/>
     </row>
     <row r="225" spans="1:17" customHeight="1" ht="15.75">
       <c r="H225" s="6"/>
-      <c r="I225" s="13"/>
+      <c r="I225" s="6"/>
     </row>
     <row r="226" spans="1:17" customHeight="1" ht="15.75">
       <c r="H226" s="6"/>
-      <c r="I226" s="13"/>
+      <c r="I226" s="6"/>
     </row>
     <row r="227" spans="1:17" customHeight="1" ht="15.75">
       <c r="H227" s="6"/>
-      <c r="I227" s="13"/>
+      <c r="I227" s="6"/>
     </row>
     <row r="228" spans="1:17" customHeight="1" ht="15.75">
       <c r="H228" s="6"/>
-      <c r="I228" s="13"/>
+      <c r="I228" s="6"/>
     </row>
     <row r="229" spans="1:17" customHeight="1" ht="15.75">
       <c r="H229" s="6"/>
-      <c r="I229" s="13"/>
+      <c r="I229" s="6"/>
     </row>
     <row r="230" spans="1:17" customHeight="1" ht="15.75">
       <c r="H230" s="6"/>
-      <c r="I230" s="13"/>
+      <c r="I230" s="6"/>
     </row>
     <row r="231" spans="1:17" customHeight="1" ht="15.75">
       <c r="H231" s="6"/>
-      <c r="I231" s="13"/>
+      <c r="I231" s="6"/>
     </row>
     <row r="232" spans="1:17" customHeight="1" ht="15.75">
       <c r="H232" s="6"/>
-      <c r="I232" s="13"/>
+      <c r="I232" s="6"/>
     </row>
     <row r="233" spans="1:17" customHeight="1" ht="15.75">
       <c r="H233" s="6"/>
-      <c r="I233" s="13"/>
+      <c r="I233" s="6"/>
     </row>
     <row r="234" spans="1:17" customHeight="1" ht="15.75">
       <c r="H234" s="6"/>
-      <c r="I234" s="13"/>
+      <c r="I234" s="6"/>
     </row>
     <row r="235" spans="1:17" customHeight="1" ht="15.75">
       <c r="H235" s="6"/>
-      <c r="I235" s="13"/>
+      <c r="I235" s="6"/>
     </row>
     <row r="236" spans="1:17" customHeight="1" ht="15.75">
       <c r="H236" s="6"/>
-      <c r="I236" s="13"/>
+      <c r="I236" s="6"/>
     </row>
     <row r="237" spans="1:17" customHeight="1" ht="15.75">
       <c r="H237" s="6"/>
-      <c r="I237" s="13"/>
+      <c r="I237" s="6"/>
     </row>
     <row r="238" spans="1:17" customHeight="1" ht="15.75">
       <c r="H238" s="6"/>
-      <c r="I238" s="13"/>
+      <c r="I238" s="6"/>
     </row>
     <row r="239" spans="1:17" customHeight="1" ht="15.75">
       <c r="H239" s="6"/>
-      <c r="I239" s="13"/>
+      <c r="I239" s="6"/>
     </row>
     <row r="240" spans="1:17" customHeight="1" ht="15.75">
       <c r="H240" s="6"/>
-      <c r="I240" s="13"/>
+      <c r="I240" s="6"/>
     </row>
     <row r="241" spans="1:17" customHeight="1" ht="15.75">
       <c r="H241" s="6"/>
-      <c r="I241" s="13"/>
+      <c r="I241" s="6"/>
     </row>
     <row r="242" spans="1:17" customHeight="1" ht="15.75">
       <c r="H242" s="6"/>
-      <c r="I242" s="13"/>
+      <c r="I242" s="6"/>
     </row>
     <row r="243" spans="1:17" customHeight="1" ht="15.75">
       <c r="H243" s="6"/>
-      <c r="I243" s="13"/>
+      <c r="I243" s="6"/>
     </row>
     <row r="244" spans="1:17" customHeight="1" ht="15.75">
       <c r="H244" s="6"/>
-      <c r="I244" s="13"/>
+      <c r="I244" s="6"/>
     </row>
     <row r="245" spans="1:17" customHeight="1" ht="15.75">
       <c r="H245" s="6"/>
-      <c r="I245" s="13"/>
+      <c r="I245" s="6"/>
     </row>
     <row r="246" spans="1:17" customHeight="1" ht="15.75">
       <c r="H246" s="6"/>
-      <c r="I246" s="13"/>
+      <c r="I246" s="6"/>
     </row>
     <row r="247" spans="1:17" customHeight="1" ht="15.75">
       <c r="H247" s="6"/>
-      <c r="I247" s="13"/>
+      <c r="I247" s="6"/>
     </row>
     <row r="248" spans="1:17" customHeight="1" ht="15.75">
       <c r="H248" s="6"/>
-      <c r="I248" s="13"/>
+      <c r="I248" s="6"/>
     </row>
     <row r="249" spans="1:17" customHeight="1" ht="15.75">
       <c r="H249" s="6"/>
-      <c r="I249" s="13"/>
+      <c r="I249" s="6"/>
     </row>
     <row r="250" spans="1:17" customHeight="1" ht="15.75">
       <c r="H250" s="6"/>
-      <c r="I250" s="13"/>
+      <c r="I250" s="6"/>
     </row>
     <row r="251" spans="1:17" customHeight="1" ht="15.75">
       <c r="H251" s="6"/>
-      <c r="I251" s="13"/>
+      <c r="I251" s="6"/>
     </row>
     <row r="252" spans="1:17" customHeight="1" ht="15.75">
       <c r="H252" s="6"/>
-      <c r="I252" s="13"/>
+      <c r="I252" s="6"/>
     </row>
     <row r="253" spans="1:17" customHeight="1" ht="15.75">
       <c r="H253" s="6"/>
-      <c r="I253" s="13"/>
+      <c r="I253" s="6"/>
     </row>
     <row r="254" spans="1:17" customHeight="1" ht="15.75">
       <c r="H254" s="6"/>
-      <c r="I254" s="13"/>
+      <c r="I254" s="6"/>
     </row>
     <row r="255" spans="1:17" customHeight="1" ht="15.75">
       <c r="H255" s="6"/>
-      <c r="I255" s="13"/>
+      <c r="I255" s="6"/>
     </row>
     <row r="256" spans="1:17" customHeight="1" ht="15.75">
       <c r="H256" s="6"/>
-      <c r="I256" s="13"/>
+      <c r="I256" s="6"/>
     </row>
     <row r="257" spans="1:17" customHeight="1" ht="15.75">
       <c r="H257" s="6"/>
-      <c r="I257" s="13"/>
+      <c r="I257" s="6"/>
     </row>
     <row r="258" spans="1:17" customHeight="1" ht="15.75">
       <c r="H258" s="6"/>
-      <c r="I258" s="13"/>
+      <c r="I258" s="6"/>
     </row>
     <row r="259" spans="1:17" customHeight="1" ht="15.75">
       <c r="H259" s="6"/>
-      <c r="I259" s="13"/>
+      <c r="I259" s="6"/>
     </row>
     <row r="260" spans="1:17" customHeight="1" ht="15.75">
       <c r="H260" s="6"/>
-      <c r="I260" s="13"/>
+      <c r="I260" s="6"/>
     </row>
     <row r="261" spans="1:17" customHeight="1" ht="15.75">
       <c r="H261" s="6"/>
-      <c r="I261" s="13"/>
+      <c r="I261" s="6"/>
     </row>
     <row r="262" spans="1:17" customHeight="1" ht="15.75">
       <c r="H262" s="6"/>
-      <c r="I262" s="13"/>
+      <c r="I262" s="6"/>
     </row>
     <row r="263" spans="1:17" customHeight="1" ht="15.75">
       <c r="H263" s="6"/>
-      <c r="I263" s="13"/>
+      <c r="I263" s="6"/>
     </row>
     <row r="264" spans="1:17" customHeight="1" ht="15.75">
       <c r="H264" s="6"/>
-      <c r="I264" s="13"/>
+      <c r="I264" s="6"/>
     </row>
     <row r="265" spans="1:17" customHeight="1" ht="15.75">
       <c r="H265" s="6"/>
-      <c r="I265" s="13"/>
+      <c r="I265" s="6"/>
     </row>
     <row r="266" spans="1:17" customHeight="1" ht="15.75">
       <c r="H266" s="6"/>
-      <c r="I266" s="13"/>
+      <c r="I266" s="6"/>
     </row>
     <row r="267" spans="1:17" customHeight="1" ht="15.75">
       <c r="H267" s="6"/>
-      <c r="I267" s="13"/>
+      <c r="I267" s="6"/>
     </row>
     <row r="268" spans="1:17" customHeight="1" ht="15.75">
       <c r="H268" s="6"/>
-      <c r="I268" s="13"/>
+      <c r="I268" s="6"/>
     </row>
     <row r="269" spans="1:17" customHeight="1" ht="15.75">
       <c r="H269" s="6"/>
-      <c r="I269" s="13"/>
+      <c r="I269" s="6"/>
     </row>
     <row r="270" spans="1:17" customHeight="1" ht="15.75">
       <c r="H270" s="6"/>
-      <c r="I270" s="13"/>
+      <c r="I270" s="6"/>
     </row>
     <row r="271" spans="1:17" customHeight="1" ht="15.75">
       <c r="H271" s="6"/>
-      <c r="I271" s="13"/>
+      <c r="I271" s="6"/>
     </row>
     <row r="272" spans="1:17" customHeight="1" ht="15.75">
       <c r="H272" s="6"/>
-      <c r="I272" s="13"/>
+      <c r="I272" s="6"/>
     </row>
     <row r="273" spans="1:17" customHeight="1" ht="15.75">
       <c r="H273" s="6"/>
-      <c r="I273" s="13"/>
+      <c r="I273" s="6"/>
     </row>
     <row r="274" spans="1:17" customHeight="1" ht="15.75">
       <c r="H274" s="6"/>
-      <c r="I274" s="13"/>
+      <c r="I274" s="6"/>
     </row>
     <row r="275" spans="1:17" customHeight="1" ht="15.75">
       <c r="H275" s="6"/>
-      <c r="I275" s="13"/>
+      <c r="I275" s="6"/>
     </row>
     <row r="276" spans="1:17" customHeight="1" ht="15.75">
       <c r="H276" s="6"/>
-      <c r="I276" s="13"/>
+      <c r="I276" s="6"/>
     </row>
     <row r="277" spans="1:17" customHeight="1" ht="15.75">
       <c r="H277" s="6"/>
-      <c r="I277" s="13"/>
+      <c r="I277" s="6"/>
     </row>
     <row r="278" spans="1:17" customHeight="1" ht="15.75">
       <c r="H278" s="6"/>
-      <c r="I278" s="13"/>
+      <c r="I278" s="6"/>
     </row>
     <row r="279" spans="1:17" customHeight="1" ht="15.75">
       <c r="H279" s="6"/>
-      <c r="I279" s="13"/>
+      <c r="I279" s="6"/>
     </row>
     <row r="280" spans="1:17" customHeight="1" ht="15.75">
       <c r="H280" s="6"/>
-      <c r="I280" s="13"/>
+      <c r="I280" s="6"/>
     </row>
     <row r="281" spans="1:17" customHeight="1" ht="15.75">
       <c r="H281" s="6"/>
-      <c r="I281" s="13"/>
+      <c r="I281" s="6"/>
     </row>
     <row r="282" spans="1:17" customHeight="1" ht="15.75">
       <c r="H282" s="6"/>
-      <c r="I282" s="13"/>
+      <c r="I282" s="6"/>
     </row>
     <row r="283" spans="1:17" customHeight="1" ht="15.75">
       <c r="H283" s="6"/>
-      <c r="I283" s="13"/>
+      <c r="I283" s="6"/>
     </row>
     <row r="284" spans="1:17" customHeight="1" ht="15.75">
       <c r="H284" s="6"/>
-      <c r="I284" s="13"/>
+      <c r="I284" s="6"/>
     </row>
     <row r="285" spans="1:17" customHeight="1" ht="15.75">
       <c r="H285" s="6"/>
-      <c r="I285" s="13"/>
+      <c r="I285" s="6"/>
     </row>
     <row r="286" spans="1:17" customHeight="1" ht="15.75">
       <c r="H286" s="6"/>
-      <c r="I286" s="13"/>
+      <c r="I286" s="6"/>
     </row>
     <row r="287" spans="1:17" customHeight="1" ht="15.75">
       <c r="H287" s="6"/>
-      <c r="I287" s="13"/>
+      <c r="I287" s="6"/>
     </row>
     <row r="288" spans="1:17" customHeight="1" ht="15.75">
       <c r="H288" s="6"/>
-      <c r="I288" s="13"/>
+      <c r="I288" s="6"/>
     </row>
     <row r="289" spans="1:17" customHeight="1" ht="15.75">
       <c r="H289" s="6"/>
-      <c r="I289" s="13"/>
+      <c r="I289" s="6"/>
     </row>
     <row r="290" spans="1:17" customHeight="1" ht="15.75">
       <c r="H290" s="6"/>
-      <c r="I290" s="13"/>
+      <c r="I290" s="6"/>
     </row>
     <row r="291" spans="1:17" customHeight="1" ht="15.75">
       <c r="H291" s="6"/>
-      <c r="I291" s="13"/>
+      <c r="I291" s="6"/>
     </row>
     <row r="292" spans="1:17" customHeight="1" ht="15.75">
       <c r="H292" s="6"/>
-      <c r="I292" s="13"/>
+      <c r="I292" s="6"/>
     </row>
     <row r="293" spans="1:17" customHeight="1" ht="15.75">
       <c r="H293" s="6"/>
-      <c r="I293" s="13"/>
+      <c r="I293" s="6"/>
     </row>
     <row r="294" spans="1:17" customHeight="1" ht="15.75">
       <c r="H294" s="6"/>
-      <c r="I294" s="13"/>
+      <c r="I294" s="6"/>
     </row>
     <row r="295" spans="1:17" customHeight="1" ht="15.75">
       <c r="H295" s="6"/>
-      <c r="I295" s="13"/>
+      <c r="I295" s="6"/>
     </row>
     <row r="296" spans="1:17" customHeight="1" ht="15.75">
       <c r="H296" s="6"/>
-      <c r="I296" s="13"/>
+      <c r="I296" s="6"/>
     </row>
     <row r="297" spans="1:17" customHeight="1" ht="15.75">
       <c r="H297" s="6"/>
-      <c r="I297" s="13"/>
+      <c r="I297" s="6"/>
     </row>
     <row r="298" spans="1:17" customHeight="1" ht="15.75">
       <c r="H298" s="6"/>
-      <c r="I298" s="13"/>
+      <c r="I298" s="6"/>
     </row>
     <row r="299" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I299" s="13"/>
+      <c r="I299" s="6"/>
     </row>
     <row r="300" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I300" s="13"/>
+      <c r="I300" s="6"/>
     </row>
     <row r="301" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I301" s="13"/>
+      <c r="I301" s="6"/>
     </row>
     <row r="302" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I302" s="13"/>
+      <c r="I302" s="6"/>
     </row>
     <row r="303" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I303" s="13"/>
+      <c r="I303" s="6"/>
     </row>
     <row r="304" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I304" s="13"/>
+      <c r="I304" s="6"/>
     </row>
     <row r="305" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I305" s="13"/>
+      <c r="I305" s="6"/>
     </row>
     <row r="306" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I306" s="13"/>
+      <c r="I306" s="6"/>
     </row>
     <row r="307" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I307" s="13"/>
+      <c r="I307" s="6"/>
     </row>
     <row r="308" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I308" s="13"/>
+      <c r="I308" s="6"/>
     </row>
     <row r="309" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I309" s="13"/>
+      <c r="I309" s="6"/>
     </row>
     <row r="310" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I310" s="13"/>
+      <c r="I310" s="6"/>
     </row>
     <row r="311" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I311" s="13"/>
+      <c r="I311" s="6"/>
     </row>
     <row r="312" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I312" s="13"/>
+      <c r="I312" s="6"/>
     </row>
     <row r="313" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I313" s="13"/>
+      <c r="I313" s="6"/>
     </row>
     <row r="314" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I314" s="13"/>
+      <c r="I314" s="6"/>
     </row>
     <row r="315" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I315" s="13"/>
+      <c r="I315" s="6"/>
     </row>
     <row r="316" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I316" s="13"/>
+      <c r="I316" s="6"/>
     </row>
     <row r="317" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I317" s="13"/>
+      <c r="I317" s="6"/>
     </row>
     <row r="318" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I318" s="13"/>
+      <c r="I318" s="6"/>
     </row>
     <row r="319" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I319" s="13"/>
+      <c r="I319" s="6"/>
     </row>
     <row r="320" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I320" s="13"/>
+      <c r="I320" s="6"/>
     </row>
     <row r="321" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I321" s="13"/>
+      <c r="I321" s="6"/>
     </row>
     <row r="322" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I322" s="13"/>
+      <c r="I322" s="6"/>
     </row>
     <row r="323" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I323" s="13"/>
+      <c r="I323" s="6"/>
     </row>
     <row r="324" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I324" s="13"/>
+      <c r="I324" s="6"/>
     </row>
     <row r="325" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I325" s="13"/>
+      <c r="I325" s="6"/>
     </row>
     <row r="326" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I326" s="13"/>
+      <c r="I326" s="6"/>
     </row>
     <row r="327" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I327" s="13"/>
+      <c r="I327" s="6"/>
     </row>
     <row r="328" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I328" s="13"/>
+      <c r="I328" s="6"/>
     </row>
     <row r="329" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I329" s="13"/>
+      <c r="I329" s="6"/>
     </row>
     <row r="330" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I330" s="13"/>
+      <c r="I330" s="6"/>
     </row>
     <row r="331" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I331" s="13"/>
+      <c r="I331" s="6"/>
     </row>
     <row r="332" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I332" s="13"/>
+      <c r="I332" s="6"/>
     </row>
     <row r="333" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I333" s="13"/>
+      <c r="I333" s="6"/>
     </row>
     <row r="334" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I334" s="13"/>
+      <c r="I334" s="6"/>
     </row>
     <row r="335" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I335" s="13"/>
+      <c r="I335" s="6"/>
     </row>
     <row r="336" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I336" s="13"/>
+      <c r="I336" s="6"/>
     </row>
     <row r="337" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I337" s="13"/>
+      <c r="I337" s="6"/>
     </row>
     <row r="338" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I338" s="13"/>
+      <c r="I338" s="6"/>
     </row>
     <row r="339" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I339" s="13"/>
+      <c r="I339" s="6"/>
     </row>
     <row r="340" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I340" s="13"/>
+      <c r="I340" s="6"/>
     </row>
     <row r="341" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I341" s="13"/>
+      <c r="I341" s="6"/>
     </row>
     <row r="342" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I342" s="13"/>
+      <c r="I342" s="6"/>
     </row>
     <row r="343" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I343" s="13"/>
+      <c r="I343" s="6"/>
     </row>
     <row r="344" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I344" s="13"/>
+      <c r="I344" s="6"/>
     </row>
     <row r="345" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I345" s="13"/>
+      <c r="I345" s="6"/>
     </row>
     <row r="346" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I346" s="13"/>
+      <c r="I346" s="6"/>
     </row>
     <row r="347" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I347" s="13"/>
+      <c r="I347" s="6"/>
     </row>
     <row r="348" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I348" s="13"/>
+      <c r="I348" s="6"/>
     </row>
     <row r="349" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I349" s="13"/>
+      <c r="I349" s="6"/>
     </row>
     <row r="350" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I350" s="13"/>
+      <c r="I350" s="6"/>
     </row>
     <row r="351" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I351" s="13"/>
+      <c r="I351" s="6"/>
     </row>
     <row r="352" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I352" s="13"/>
+      <c r="I352" s="6"/>
     </row>
     <row r="353" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I353" s="13"/>
+      <c r="I353" s="6"/>
     </row>
     <row r="354" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I354" s="13"/>
+      <c r="I354" s="6"/>
     </row>
     <row r="355" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I355" s="13"/>
+      <c r="I355" s="6"/>
     </row>
     <row r="356" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I356" s="13"/>
+      <c r="I356" s="6"/>
     </row>
     <row r="357" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I357" s="13"/>
+      <c r="I357" s="6"/>
     </row>
     <row r="358" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I358" s="13"/>
+      <c r="I358" s="6"/>
     </row>
     <row r="359" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I359" s="13"/>
+      <c r="I359" s="6"/>
     </row>
     <row r="360" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I360" s="13"/>
+      <c r="I360" s="6"/>
     </row>
     <row r="361" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I361" s="13"/>
+      <c r="I361" s="6"/>
     </row>
     <row r="362" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I362" s="13"/>
+      <c r="I362" s="6"/>
     </row>
     <row r="363" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I363" s="13"/>
+      <c r="I363" s="6"/>
     </row>
     <row r="364" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I364" s="13"/>
+      <c r="I364" s="6"/>
     </row>
     <row r="365" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I365" s="13"/>
+      <c r="I365" s="6"/>
     </row>
     <row r="366" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I366" s="13"/>
+      <c r="I366" s="6"/>
     </row>
     <row r="367" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I367" s="13"/>
+      <c r="I367" s="6"/>
     </row>
     <row r="368" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I368" s="13"/>
+      <c r="I368" s="6"/>
     </row>
     <row r="369" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I369" s="13"/>
+      <c r="I369" s="6"/>
     </row>
     <row r="370" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I370" s="13"/>
+      <c r="I370" s="6"/>
     </row>
     <row r="371" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I371" s="13"/>
+      <c r="I371" s="6"/>
     </row>
     <row r="372" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I372" s="13"/>
+      <c r="I372" s="6"/>
     </row>
     <row r="373" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I373" s="13"/>
+      <c r="I373" s="6"/>
     </row>
     <row r="374" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I374" s="13"/>
+      <c r="I374" s="6"/>
     </row>
     <row r="375" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I375" s="13"/>
+      <c r="I375" s="6"/>
     </row>
     <row r="376" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I376" s="13"/>
+      <c r="I376" s="6"/>
     </row>
     <row r="377" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I377" s="13"/>
+      <c r="I377" s="6"/>
     </row>
     <row r="378" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I378" s="13"/>
+      <c r="I378" s="6"/>
     </row>
     <row r="379" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I379" s="13"/>
+      <c r="I379" s="6"/>
     </row>
     <row r="380" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I380" s="13"/>
+      <c r="I380" s="6"/>
     </row>
     <row r="381" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I381" s="13"/>
+      <c r="I381" s="6"/>
     </row>
     <row r="382" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I382" s="13"/>
+      <c r="I382" s="6"/>
     </row>
     <row r="383" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I383" s="13"/>
+      <c r="I383" s="6"/>
     </row>
     <row r="384" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I384" s="13"/>
+      <c r="I384" s="6"/>
     </row>
     <row r="385" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I385" s="13"/>
+      <c r="I385" s="6"/>
     </row>
     <row r="386" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I386" s="13"/>
+      <c r="I386" s="6"/>
     </row>
     <row r="387" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I387" s="13"/>
+      <c r="I387" s="6"/>
     </row>
     <row r="388" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I388" s="13"/>
+      <c r="I388" s="6"/>
     </row>
     <row r="389" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I389" s="13"/>
+      <c r="I389" s="6"/>
     </row>
     <row r="390" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I390" s="13"/>
+      <c r="I390" s="6"/>
     </row>
     <row r="391" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I391" s="13"/>
+      <c r="I391" s="6"/>
     </row>
     <row r="392" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I392" s="13"/>
+      <c r="I392" s="6"/>
     </row>
     <row r="393" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I393" s="13"/>
+      <c r="I393" s="6"/>
     </row>
     <row r="394" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I394" s="13"/>
+      <c r="I394" s="6"/>
     </row>
     <row r="395" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I395" s="13"/>
+      <c r="I395" s="6"/>
     </row>
     <row r="396" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I396" s="13"/>
+      <c r="I396" s="6"/>
     </row>
     <row r="397" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I397" s="13"/>
+      <c r="I397" s="6"/>
     </row>
     <row r="398" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I398" s="13"/>
+      <c r="I398" s="6"/>
     </row>
     <row r="399" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I399" s="13"/>
+      <c r="I399" s="6"/>
     </row>
     <row r="400" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I400" s="13"/>
+      <c r="I400" s="6"/>
     </row>
     <row r="401" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I401" s="13"/>
+      <c r="I401" s="6"/>
     </row>
     <row r="402" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I402" s="13"/>
+      <c r="I402" s="6"/>
     </row>
     <row r="403" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I403" s="13"/>
+      <c r="I403" s="6"/>
     </row>
     <row r="404" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I404" s="13"/>
+      <c r="I404" s="6"/>
     </row>
     <row r="405" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I405" s="13"/>
+      <c r="I405" s="6"/>
     </row>
     <row r="406" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I406" s="13"/>
+      <c r="I406" s="6"/>
     </row>
     <row r="407" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I407" s="13"/>
+      <c r="I407" s="6"/>
     </row>
     <row r="408" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I408" s="13"/>
+      <c r="I408" s="6"/>
     </row>
     <row r="409" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I409" s="13"/>
+      <c r="I409" s="6"/>
     </row>
     <row r="410" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I410" s="13"/>
+      <c r="I410" s="6"/>
     </row>
     <row r="411" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I411" s="13"/>
+      <c r="I411" s="6"/>
     </row>
     <row r="412" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I412" s="13"/>
+      <c r="I412" s="6"/>
     </row>
     <row r="413" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I413" s="13"/>
+      <c r="I413" s="6"/>
     </row>
     <row r="414" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I414" s="13"/>
+      <c r="I414" s="6"/>
     </row>
     <row r="415" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I415" s="13"/>
+      <c r="I415" s="6"/>
     </row>
     <row r="416" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I416" s="13"/>
+      <c r="I416" s="6"/>
     </row>
     <row r="417" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I417" s="13"/>
+      <c r="I417" s="6"/>
     </row>
     <row r="418" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I418" s="13"/>
+      <c r="I418" s="6"/>
     </row>
     <row r="419" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I419" s="13"/>
+      <c r="I419" s="6"/>
     </row>
     <row r="420" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I420" s="13"/>
+      <c r="I420" s="6"/>
     </row>
     <row r="421" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I421" s="13"/>
+      <c r="I421" s="6"/>
     </row>
     <row r="422" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I422" s="13"/>
+      <c r="I422" s="6"/>
     </row>
     <row r="423" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I423" s="13"/>
+      <c r="I423" s="6"/>
     </row>
     <row r="424" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I424" s="13"/>
+      <c r="I424" s="6"/>
     </row>
     <row r="425" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I425" s="13"/>
+      <c r="I425" s="6"/>
     </row>
     <row r="426" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I426" s="13"/>
+      <c r="I426" s="6"/>
     </row>
     <row r="427" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I427" s="13"/>
+      <c r="I427" s="6"/>
     </row>
     <row r="428" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I428" s="13"/>
+      <c r="I428" s="6"/>
     </row>
     <row r="429" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I429" s="13"/>
+      <c r="I429" s="6"/>
     </row>
     <row r="430" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I430" s="13"/>
+      <c r="I430" s="6"/>
     </row>
     <row r="431" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I431" s="13"/>
+      <c r="I431" s="6"/>
     </row>
     <row r="432" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I432" s="13"/>
+      <c r="I432" s="6"/>
     </row>
     <row r="433" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I433" s="13"/>
+      <c r="I433" s="6"/>
     </row>
     <row r="434" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I434" s="13"/>
+      <c r="I434" s="6"/>
     </row>
     <row r="435" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I435" s="13"/>
+      <c r="I435" s="6"/>
     </row>
     <row r="436" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I436" s="13"/>
+      <c r="I436" s="6"/>
     </row>
     <row r="437" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I437" s="13"/>
+      <c r="I437" s="6"/>
     </row>
     <row r="438" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I438" s="13"/>
+      <c r="I438" s="6"/>
     </row>
     <row r="439" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I439" s="13"/>
+      <c r="I439" s="6"/>
     </row>
     <row r="440" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I440" s="13"/>
+      <c r="I440" s="6"/>
     </row>
     <row r="441" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I441" s="13"/>
+      <c r="I441" s="6"/>
     </row>
     <row r="442" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I442" s="13"/>
+      <c r="I442" s="6"/>
     </row>
     <row r="443" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I443" s="13"/>
+      <c r="I443" s="6"/>
     </row>
     <row r="444" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I444" s="13"/>
+      <c r="I444" s="6"/>
     </row>
     <row r="445" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I445" s="13"/>
+      <c r="I445" s="6"/>
     </row>
     <row r="446" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I446" s="13"/>
+      <c r="I446" s="6"/>
     </row>
     <row r="447" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I447" s="13"/>
+      <c r="I447" s="6"/>
     </row>
     <row r="448" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I448" s="13"/>
+      <c r="I448" s="6"/>
     </row>
     <row r="449" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I449" s="13"/>
+      <c r="I449" s="6"/>
     </row>
     <row r="450" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I450" s="13"/>
+      <c r="I450" s="6"/>
     </row>
     <row r="451" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I451" s="13"/>
+      <c r="I451" s="6"/>
     </row>
     <row r="452" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I452" s="13"/>
+      <c r="I452" s="6"/>
     </row>
     <row r="453" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I453" s="13"/>
+      <c r="I453" s="6"/>
     </row>
     <row r="454" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I454" s="13"/>
+      <c r="I454" s="6"/>
     </row>
     <row r="455" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I455" s="13"/>
+      <c r="I455" s="6"/>
     </row>
     <row r="456" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I456" s="13"/>
+      <c r="I456" s="6"/>
     </row>
     <row r="457" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I457" s="13"/>
+      <c r="I457" s="6"/>
     </row>
     <row r="458" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I458" s="13"/>
+      <c r="I458" s="6"/>
     </row>
     <row r="459" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I459" s="13"/>
+      <c r="I459" s="6"/>
     </row>
     <row r="460" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I460" s="13"/>
+      <c r="I460" s="6"/>
     </row>
     <row r="461" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I461" s="13"/>
+      <c r="I461" s="6"/>
     </row>
     <row r="462" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I462" s="13"/>
+      <c r="I462" s="6"/>
     </row>
     <row r="463" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I463" s="13"/>
+      <c r="I463" s="6"/>
     </row>
     <row r="464" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I464" s="13"/>
+      <c r="I464" s="6"/>
     </row>
     <row r="465" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I465" s="13"/>
+      <c r="I465" s="6"/>
     </row>
     <row r="466" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I466" s="13"/>
+      <c r="I466" s="6"/>
     </row>
     <row r="467" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I467" s="13"/>
+      <c r="I467" s="6"/>
     </row>
     <row r="468" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I468" s="13"/>
+      <c r="I468" s="6"/>
     </row>
     <row r="469" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I469" s="13"/>
+      <c r="I469" s="6"/>
     </row>
     <row r="470" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I470" s="13"/>
+      <c r="I470" s="6"/>
     </row>
     <row r="471" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I471" s="13"/>
+      <c r="I471" s="6"/>
     </row>
     <row r="472" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I472" s="13"/>
+      <c r="I472" s="6"/>
     </row>
     <row r="473" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I473" s="13"/>
+      <c r="I473" s="6"/>
     </row>
     <row r="474" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I474" s="13"/>
+      <c r="I474" s="6"/>
     </row>
     <row r="475" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I475" s="13"/>
+      <c r="I475" s="6"/>
     </row>
     <row r="476" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I476" s="13"/>
+      <c r="I476" s="6"/>
     </row>
     <row r="477" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I477" s="13"/>
+      <c r="I477" s="6"/>
     </row>
     <row r="478" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I478" s="13"/>
+      <c r="I478" s="6"/>
     </row>
     <row r="479" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I479" s="13"/>
+      <c r="I479" s="6"/>
     </row>
     <row r="480" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I480" s="13"/>
+      <c r="I480" s="6"/>
     </row>
     <row r="481" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I481" s="13"/>
+      <c r="I481" s="6"/>
     </row>
     <row r="482" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I482" s="13"/>
+      <c r="I482" s="6"/>
     </row>
     <row r="483" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I483" s="13"/>
+      <c r="I483" s="6"/>
     </row>
     <row r="484" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I484" s="13"/>
+      <c r="I484" s="6"/>
     </row>
     <row r="485" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I485" s="13"/>
+      <c r="I485" s="6"/>
     </row>
     <row r="486" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I486" s="13"/>
+      <c r="I486" s="6"/>
     </row>
     <row r="487" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I487" s="13"/>
+      <c r="I487" s="6"/>
     </row>
     <row r="488" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I488" s="13"/>
+      <c r="I488" s="6"/>
     </row>
     <row r="489" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I489" s="13"/>
+      <c r="I489" s="6"/>
     </row>
     <row r="490" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I490" s="13"/>
+      <c r="I490" s="6"/>
     </row>
     <row r="491" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I491" s="13"/>
+      <c r="I491" s="6"/>
     </row>
     <row r="492" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I492" s="13"/>
+      <c r="I492" s="6"/>
     </row>
     <row r="493" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I493" s="13"/>
+      <c r="I493" s="6"/>
     </row>
     <row r="494" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I494" s="13"/>
+      <c r="I494" s="6"/>
     </row>
     <row r="495" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I495" s="13"/>
+      <c r="I495" s="6"/>
     </row>
     <row r="496" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I496" s="13"/>
+      <c r="I496" s="6"/>
     </row>
     <row r="497" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I497" s="13"/>
+      <c r="I497" s="6"/>
     </row>
     <row r="498" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I498" s="13"/>
+      <c r="I498" s="6"/>
     </row>
     <row r="499" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I499" s="13"/>
+      <c r="I499" s="6"/>
     </row>
     <row r="500" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I500" s="13"/>
+      <c r="I500" s="6"/>
     </row>
     <row r="501" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I501" s="13"/>
+      <c r="I501" s="6"/>
     </row>
     <row r="502" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I502" s="13"/>
+      <c r="I502" s="6"/>
     </row>
     <row r="503" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I503" s="13"/>
+      <c r="I503" s="6"/>
     </row>
     <row r="504" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I504" s="13"/>
+      <c r="I504" s="6"/>
     </row>
     <row r="505" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I505" s="13"/>
+      <c r="I505" s="6"/>
     </row>
     <row r="506" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I506" s="13"/>
+      <c r="I506" s="6"/>
     </row>
     <row r="507" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I507" s="13"/>
+      <c r="I507" s="6"/>
     </row>
     <row r="508" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I508" s="13"/>
+      <c r="I508" s="6"/>
     </row>
     <row r="509" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I509" s="13"/>
+      <c r="I509" s="6"/>
     </row>
     <row r="510" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I510" s="13"/>
+      <c r="I510" s="6"/>
     </row>
     <row r="511" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I511" s="13"/>
+      <c r="I511" s="6"/>
     </row>
     <row r="512" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I512" s="13"/>
+      <c r="I512" s="6"/>
     </row>
     <row r="513" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I513" s="13"/>
+      <c r="I513" s="6"/>
     </row>
     <row r="514" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I514" s="13"/>
+      <c r="I514" s="6"/>
     </row>
     <row r="515" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I515" s="13"/>
+      <c r="I515" s="6"/>
     </row>
     <row r="516" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I516" s="13"/>
+      <c r="I516" s="6"/>
     </row>
     <row r="517" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I517" s="13"/>
+      <c r="I517" s="6"/>
     </row>
     <row r="518" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I518" s="13"/>
+      <c r="I518" s="6"/>
     </row>
     <row r="519" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I519" s="13"/>
+      <c r="I519" s="6"/>
     </row>
     <row r="520" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I520" s="13"/>
+      <c r="I520" s="6"/>
     </row>
     <row r="521" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I521" s="13"/>
+      <c r="I521" s="6"/>
     </row>
     <row r="522" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I522" s="13"/>
+      <c r="I522" s="6"/>
     </row>
     <row r="523" spans="1:17" customHeight="1" ht="15.75">
-      <c r="I523" s="13"/>
+      <c r="I523" s="6"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>

</xml_diff>